<commit_message>
Filtre liste agences: garde agences classiques et réseaux de mandataires
Retire conseillers en gestion de patrimoine, experts/expertise, viager,
conciergerie/location saisonnière, gestion locative pure et promoteurs
(7 lignes supprimées, 72 restantes).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwT51bbn2dC8Mqx4ryJ3FX
</commit_message>
<xml_diff>
--- a/agences_immobilieres_mobiles.xlsx
+++ b/agences_immobilieres_mobiles.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Agences mobiles 06-07" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences mobiles 06-07'!$A$1:$E$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences mobiles 06-07'!$A$1:$E$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1111,17 +1111,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>ALPHINO Conciergerie</t>
+          <t>Coraline - La P'tite Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Hugues-Alexandre Douvesy</t>
+          <t>Coraline</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>06 68 02 73 80</t>
+          <t>06 69 60 31 52</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Coraline - La P'tite Halle de l'Immobilier</t>
+          <t>David Doizon - iad France</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Coraline</t>
+          <t>David Doizon</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>06 69 60 31 52</t>
+          <t>06 24 39 27 36</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1165,17 +1165,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>David Doizon - iad France</t>
+          <t>Florian - La P'tite Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>David Doizon</t>
+          <t>Florian</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>06 24 39 27 36</t>
+          <t>06 77 11 43 24</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1192,17 +1192,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Florian - La P'tite Halle de l'Immobilier</t>
+          <t>Henri Ardant - SAFTI</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Florian</t>
+          <t>Henri Ardant</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>06 77 11 43 24</t>
+          <t>06 73 37 27 27</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Henri Ardant - SAFTI</t>
+          <t>Julien BAPTISTE</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Henri Ardant</t>
+          <t>Julien Baptiste</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>06 73 37 27 27</t>
+          <t>06 50 72 65 48</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Julien BAPTISTE</t>
+          <t>Mathieu Royer Immobilier</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Julien Baptiste</t>
+          <t>Mathieu Royer</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>06 50 72 65 48</t>
+          <t>07 70 37 65 00</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1273,17 +1273,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Mathieu Royer Immobilier</t>
+          <t>Mathilde MARTIN - La Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Mathieu Royer</t>
+          <t>Mathilde Martin</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>07 70 37 65 00</t>
+          <t>06 29 78 02 33</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1300,17 +1300,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Mathilde MARTIN - La Halle de l'Immobilier</t>
+          <t>Stéphanie Chissadon - Optimhome</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Mathilde Martin</t>
+          <t>Stéphanie Chissadon</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>06 29 78 02 33</t>
+          <t>06 85 02 76 46</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1327,17 +1327,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Stéphanie Chissadon - Optimhome</t>
+          <t>Théau Silbermann</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Stéphanie Chissadon</t>
+          <t>Théau Silbermann</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>06 85 02 76 46</t>
+          <t>06 11 82 71 28</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1354,17 +1354,17 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Théau Silbermann</t>
+          <t>Véronique Mondon - iad France</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Théau Silbermann</t>
+          <t>Véronique Mondon</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>06 11 82 71 28</t>
+          <t>06 77 92 28 12</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1376,22 +1376,22 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Véronique Mondon - iad France</t>
+          <t>Aurelien CENCI - IAD France</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Véronique Mondon</t>
+          <t>Aurélien Cenci</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>06 77 92 28 12</t>
+          <t>06 26 44 64 05</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -1408,17 +1408,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Aurelien CENCI - IAD France</t>
+          <t>Delaporte Immobilier</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Aurélien Cenci</t>
+          <t>Aurélien Delaporte</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>06 26 44 64 05</t>
+          <t>06 19 48 20 93</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Conciergerie Amiens Loc-immo</t>
+          <t>e-mobilier Amiens</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Vivien Demarest-Gausson</t>
+          <t>S. Benarous (agent)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>06 10 16 05 79</t>
+          <t>06 35 22 43 99</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -1462,17 +1462,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Delaporte Immobilier</t>
+          <t>ESPACE &amp; WALL</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Aurélien Delaporte</t>
+          <t>Émilie Wolinne (Présidente)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>06 19 48 20 93</t>
+          <t>06 85 72 68 51</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -1489,17 +1489,17 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>e-mobilier Amiens</t>
+          <t>Estelle Desnain - Conseiller immobilier</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>S. Benarous (agent)</t>
+          <t>Estelle Desnain</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>06 35 22 43 99</t>
+          <t>06 10 93 58 83</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -1516,17 +1516,17 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>ESPACE &amp; WALL</t>
+          <t>Foudhil DAOUDI - EXPERTIMO</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Émilie Wolinne (Présidente)</t>
+          <t>Foudhil Daoudi</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>06 85 72 68 51</t>
+          <t>06 64 16 11 21</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -1543,17 +1543,17 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Estelle Desnain - Conseiller immobilier</t>
+          <t>Gregory Mattens (BSK Immobilier)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Estelle Desnain</t>
+          <t>Gregory Mattens</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>06 10 93 58 83</t>
+          <t>06 63 69 65 00</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Foudhil DAOUDI - EXPERTIMO</t>
+          <t>Hugo DUFOUR - iad Immobilier</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Foudhil Daoudi</t>
+          <t>Hugo Dufour</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>06 64 16 11 21</t>
+          <t>06 25 82 22 60</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>France EDL Amiens</t>
+          <t>Isabelle BOHAIN - IAD France</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Isabelle Bohain</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>06 01 59 17 96</t>
+          <t>06 69 51 10 53</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Gregory Mattens (BSK Immobilier)</t>
+          <t>Jérôme BAILLET - IAD France</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Gregory Mattens</t>
+          <t>Jérôme Baillet</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>06 63 69 65 00</t>
+          <t>06 81 42 56 26</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -1651,17 +1651,17 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Hugo DUFOUR - iad Immobilier</t>
+          <t>Quinet Nicolas</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Hugo Dufour</t>
+          <t>Nicolas Quinet</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>06 25 82 22 60</t>
+          <t>06 28 74 00 81</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -1678,17 +1678,17 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Isabelle BOHAIN - IAD France</t>
+          <t>Sophie Hardy Immobilier</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Isabelle Bohain</t>
+          <t>Sophie Hardy</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>06 69 51 10 53</t>
+          <t>06 79 07 80 19</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -1705,17 +1705,17 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Jérôme BAILLET - IAD France</t>
+          <t>Stéphane DEBEAUVAIS - IAD</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Jérôme Baillet</t>
+          <t>Stéphane Debeauvais</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>06 81 42 56 26</t>
+          <t>06 21 38 83 15</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -1732,17 +1732,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Quinet Nicolas</t>
+          <t>Sylvie Dieu - IAD France</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Nicolas Quinet</t>
+          <t>Sylvie Dieu</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>06 28 74 00 81</t>
+          <t>07 81 31 35 43</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -1759,17 +1759,17 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Sophie Hardy Immobilier</t>
+          <t>VERDIER Immobilier (Le Centre Immobilier)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Sophie Hardy</t>
+          <t>Nicolas Verdier</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>06 79 07 80 19</t>
+          <t>06 75 21 21 69</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -1781,103 +1781,103 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Stéphane DEBEAUVAIS - IAD</t>
+          <t>Agence immobilière 360° à Angers</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Stéphane Debeauvais</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>06 21 38 83 15</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 12 66 56 83</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Sylvie Dieu - IAD France</t>
+          <t>Le bon agent immobilier Angers</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Sylvie Dieu</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>07 81 31 35 43</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 11 51 51 87</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>VERDIER Immobilier (Le Centre Immobilier)</t>
+          <t>SDSIMMO L'AGENCE</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Nicolas Verdier</t>
+          <t>Antoine Fauché (Président)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>06 75 21 21 69</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 77 25 24 83</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Agence immobilière 360° à Angers</t>
+          <t>Agence ICImmobilier</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Jean-Marc Eisenbach</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>06 12 66 56 83</t>
+          <t>06 87 45 16 27</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -1889,22 +1889,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Bed I Home</t>
+          <t>Agence Pascale Louis Immobilier</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Pascale Louis</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>06 45 42 42 97</t>
+          <t>06 07 25 76 74</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -1916,22 +1916,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Le bon agent immobilier Angers</t>
+          <t>Logimmo Conseil</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Aurélie Bernardet</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>06 11 51 51 87</t>
+          <t>06 52 49 18 58</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -1943,22 +1943,22 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>SDSIMMO L'AGENCE</t>
+          <t>Manada Immobilier</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Antoine Fauché (Président)</t>
+          <t>Marine &amp; Julie Fananas</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>06 77 25 24 83</t>
+          <t>06 58 04 00 29</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -1970,22 +1970,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Agence ICImmobilier</t>
+          <t>Immo en Somme</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Jean-Marc Eisenbach</t>
+          <t>Anthony Mortas</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>06 87 45 16 27</t>
+          <t>06 15 01 61 62</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -1997,22 +1997,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Agence Pascale Louis Immobilier</t>
+          <t>Josse Pelletier Immobilier</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Pascale Louis</t>
+          <t>Sébastien Josse &amp; Isabelle Pelletier</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>06 07 25 76 74</t>
+          <t>06 67 27 80 80</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2024,22 +2024,22 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Logimmo Conseil</t>
+          <t>Satisfimmo</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Aurélie Bernardet</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>06 52 49 18 58</t>
+          <t>06 15 35 62 54</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2051,22 +2051,22 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Manada Immobilier</t>
+          <t>Toit pour toi</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Marine &amp; Julie Fananas</t>
+          <t>Michel Amarens</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>06 58 04 00 29</t>
+          <t>07 67 07 19 08</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2078,93 +2078,93 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Conciergerie Amiens - GET IMMO</t>
+          <t>IMMO PROFESSIONNEL</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Gaëtan Herpson</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>06 61 38 95 93</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 52 52 58 84</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Immo en Somme</t>
+          <t>Sylvain - Les Arènes Immobilier</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Anthony Mortas</t>
+          <t>Sylvain (négociateur)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>06 15 01 61 62</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 62 95 93 80</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Josse Pelletier Immobilier</t>
+          <t>Agence Estia Immobilier</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Sébastien Josse &amp; Isabelle Pelletier</t>
+          <t>Caroline Florance</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>06 67 27 80 80</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 63 79 66 76</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Satisfimmo</t>
+          <t>HOME</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2174,61 +2174,61 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>06 15 35 62 54</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 07 49 43 37</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Toit pour toi</t>
+          <t>AAlivImmo (A. Alivi Immo)</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Michel Amarens</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>07 67 07 19 08</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 19 77 10 66</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>CHARLEOS - Investissement immobilier</t>
+          <t>Agence La Locale Limoges</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Frédérick Tailpied</t>
+          <t>Julien Ribierre &amp; Dylan Di Nato</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>07 49 30 13 63</t>
+          <t>06 12 19 81 65</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
@@ -2240,22 +2240,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>IMMO PROFESSIONNEL</t>
+          <t>Julien Beauzetier (La Halle de l'Immobilier)</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Julien Beauzetier</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>06 52 52 58 84</t>
+          <t>06 11 09 74 89</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -2267,22 +2267,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Sylvain - Les Arènes Immobilier</t>
+          <t>Mélodie Garcia - La Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Sylvain (négociateur)</t>
+          <t>Mélodie Garcia</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>06 62 95 93 80</t>
+          <t>06 95 70 17 07</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -2294,22 +2294,22 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Agence Estia Immobilier</t>
+          <t>Nouveaux Horizons - Immobilier</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Caroline Florance</t>
+          <t>Romain Bardon</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>06 63 79 66 76</t>
+          <t>06 17 86 76 26</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
@@ -2321,22 +2321,22 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>CÔME Gestion</t>
+          <t>ROMAIN TERRAL</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Pauline Chevallier</t>
+          <t>Romain Terral</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>06 69 44 20 67</t>
+          <t>06 40 92 22 95</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
@@ -2348,22 +2348,22 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>Véronique QUEYREIX</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Véronique Queyreix</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>06 07 49 43 37</t>
+          <t>06 20 88 58 23</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
@@ -2375,22 +2375,22 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>AAlivImmo (A. Alivi Immo)</t>
+          <t>Cabinet Immobilier Amiénois</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Romain Hecquet (Président)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>06 19 77 10 66</t>
+          <t>06 24 21 58 52</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
@@ -2402,22 +2402,22 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Agence La Locale Limoges</t>
+          <t>HAUTS DE FRANCE IMMOBILIER</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Julien Ribierre &amp; Dylan Di Nato</t>
+          <t>Lilian Cléry (Président)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>06 12 19 81 65</t>
+          <t>06 08 51 24 30</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
@@ -2429,22 +2429,22 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Julien Beauzetier (La Halle de l'Immobilier)</t>
+          <t>SNG Amiens</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Julien Beauzetier</t>
+          <t>Jérôme Vangrevelynghe (conseiller)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>06 11 09 74 89</t>
+          <t>06 79 22 09 64</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
@@ -2453,197 +2453,8 @@
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>Mélodie Garcia - La Halle de l'Immobilier</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>Mélodie Garcia</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>06 95 70 17 07</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>Nouveaux Horizons - Immobilier</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>Romain Bardon</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>06 17 86 76 26</t>
-        </is>
-      </c>
-      <c r="E75" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>ROMAIN TERRAL</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>Romain Terral</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>06 40 92 22 95</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>Véronique QUEYREIX</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>Véronique Queyreix</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>06 20 88 58 23</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>Cabinet Immobilier Amiénois</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>Romain Hecquet (Président)</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>06 24 21 58 52</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>HAUTS DE FRANCE IMMOBILIER</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>Lilian Cléry (Président)</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>06 08 51 24 30</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>SNG Amiens</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>Jérôme Vangrevelynghe (conseiller)</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>06 79 22 09 64</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E80"/>
+  <autoFilter ref="A1:E73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Retire chasseur immobilier et conseillers independants de la liste
Garde agences classiques + reseaux de mandataires (IAD, SAFTI, Optimhome,
BSK, EXPERTIMO). 6 lignes retirees, 66 restantes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwT51bbn2dC8Mqx4ryJ3FX
</commit_message>
<xml_diff>
--- a/agences_immobilieres_mobiles.xlsx
+++ b/agences_immobilieres_mobiles.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Agences mobiles 06-07" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences mobiles 06-07'!$A$1:$E$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences mobiles 06-07'!$A$1:$E$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -544,17 +544,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Eric JERBRON Conseiller immobilier</t>
+          <t>Estimation Immobilière offerte à Angers</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Eric Jerbron</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>06 51 67 28 20</t>
+          <t>07 68 02 79 28</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -571,17 +571,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Estelle Payraudeau - Mon Chasseur Immo</t>
+          <t>KARACTERRE</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Estelle Payraudeau</t>
+          <t>Guillaume Sauvestre (Huby-Sauvestre)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>06 80 64 33 05</t>
+          <t>06 38 44 56 19</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -598,17 +598,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Estimation Immobilière offerte à Angers</t>
+          <t>Les Arènes Immobilier</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Victor Carme</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>07 68 02 79 28</t>
+          <t>06 46 18 29 29</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -625,17 +625,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>KARACTERRE</t>
+          <t>Maryline DELAHAYE Immobilier</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Guillaume Sauvestre (Huby-Sauvestre)</t>
+          <t>Maryline Delahaye (agent indép.)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>06 38 44 56 19</t>
+          <t>06 63 25 30 84</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -652,17 +652,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Les Arènes Immobilier</t>
+          <t>Terre d'Anjou</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Victor Carme</t>
+          <t>Anne Saison</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>06 46 18 29 29</t>
+          <t>06 19 34 36 34</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -674,22 +674,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Maryline DELAHAYE Immobilier</t>
+          <t>Barbas Immobilier</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Maryline Delahaye (agent indép.)</t>
+          <t>Anthony Barbas</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>06 63 25 30 84</t>
+          <t>06 66 73 03 71</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -701,22 +701,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Terre d'Anjou</t>
+          <t>Cabinet Blique</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Anne Saison</t>
+          <t>Charles-Adrien Blique</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>06 19 34 36 34</t>
+          <t>06 31 60 95 79</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -733,17 +733,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Barbas Immobilier</t>
+          <t>ELYX</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Anthony Barbas</t>
+          <t>Non confirmé sur Pappers</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>06 66 73 03 71</t>
+          <t>07 84 11 57 77</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -760,17 +760,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cabinet Blique</t>
+          <t>Emilie Joly - Immobilier Nancy</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Charles-Adrien Blique</t>
+          <t>Emilie Joly</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>06 31 60 95 79</t>
+          <t>06 79 55 99 77</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -787,17 +787,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ELYX</t>
+          <t>François Cossin - SAFTI</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Non confirmé sur Pappers</t>
+          <t>François Cossin</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>07 84 11 57 77</t>
+          <t>06 72 85 13 08</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -814,17 +814,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Emilie Joly - Immobilier Nancy</t>
+          <t>L'Hôtel Immobilier</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Emilie Joly</t>
+          <t>Arnaud Giacomoni</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>06 79 55 99 77</t>
+          <t>06 70 94 78 65</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -841,17 +841,17 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>François Cossin - SAFTI</t>
+          <t>Malherbe Immobilier</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>François Cossin</t>
+          <t>Vincent Malherbe</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>06 72 85 13 08</t>
+          <t>06 35 55 33 64</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -868,17 +868,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>L'Hôtel Immobilier</t>
+          <t>Paul WAGNER - SAFTI</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Arnaud Giacomoni</t>
+          <t>Paul Wagner</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>06 70 94 78 65</t>
+          <t>06 29 16 22 48</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -895,17 +895,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Malherbe Immobilier</t>
+          <t>Perlimmo</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Vincent Malherbe</t>
+          <t>Laurent Contal</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>06 35 55 33 64</t>
+          <t>06 61 22 05 74</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -922,17 +922,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Paul WAGNER - SAFTI</t>
+          <t>RODRIGUES Immobilier</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Paul Wagner</t>
+          <t>Arthur Rodrigues</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>06 29 16 22 48</t>
+          <t>07 83 04 91 26</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -949,17 +949,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Perlimmo</t>
+          <t>Signatures Immobilier</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Laurent Contal</t>
+          <t>Caroline Didelot</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>06 61 22 05 74</t>
+          <t>07 67 29 20 08</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -971,22 +971,22 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>RODRIGUES Immobilier</t>
+          <t>Adrien TRIBOULET</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Arthur Rodrigues</t>
+          <t>Adrien Triboulet</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>07 83 04 91 26</t>
+          <t>06 59 53 15 86</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -998,22 +998,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Signatures Immobilier</t>
+          <t>Agence Immobilière Celaur</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Caroline Didelot</t>
+          <t>Clément Charmes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>07 67 29 20 08</t>
+          <t>06 72 62 09 05</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Adrien TRIBOULET</t>
+          <t>Agence Première Ligne</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Adrien Triboulet</t>
+          <t>Nathalie &amp; Jean-Marie Maindrou</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>06 59 53 15 86</t>
+          <t>06 21 53 09 74</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1057,17 +1057,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Agence Immobilière Celaur</t>
+          <t>Coraline - La P'tite Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Clément Charmes</t>
+          <t>Coraline</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>06 72 62 09 05</t>
+          <t>06 69 60 31 52</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1084,17 +1084,17 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Agence Première Ligne</t>
+          <t>David Doizon - iad France</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Nathalie &amp; Jean-Marie Maindrou</t>
+          <t>David Doizon</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>06 21 53 09 74</t>
+          <t>06 24 39 27 36</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Coraline - La P'tite Halle de l'Immobilier</t>
+          <t>Florian - La P'tite Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Coraline</t>
+          <t>Florian</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>06 69 60 31 52</t>
+          <t>06 77 11 43 24</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>David Doizon - iad France</t>
+          <t>Henri Ardant - SAFTI</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>David Doizon</t>
+          <t>Henri Ardant</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>06 24 39 27 36</t>
+          <t>06 73 37 27 27</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1165,17 +1165,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Florian - La P'tite Halle de l'Immobilier</t>
+          <t>Julien BAPTISTE</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Florian</t>
+          <t>Julien Baptiste</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>06 77 11 43 24</t>
+          <t>06 50 72 65 48</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1192,17 +1192,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Henri Ardant - SAFTI</t>
+          <t>Mathieu Royer Immobilier</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Henri Ardant</t>
+          <t>Mathieu Royer</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>06 73 37 27 27</t>
+          <t>07 70 37 65 00</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Julien BAPTISTE</t>
+          <t>Mathilde MARTIN - La Halle de l'Immobilier</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Julien Baptiste</t>
+          <t>Mathilde Martin</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>06 50 72 65 48</t>
+          <t>06 29 78 02 33</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Mathieu Royer Immobilier</t>
+          <t>Stéphanie Chissadon - Optimhome</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Mathieu Royer</t>
+          <t>Stéphanie Chissadon</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>07 70 37 65 00</t>
+          <t>06 85 02 76 46</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1273,17 +1273,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Mathilde MARTIN - La Halle de l'Immobilier</t>
+          <t>Théau Silbermann</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Mathilde Martin</t>
+          <t>Théau Silbermann</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>06 29 78 02 33</t>
+          <t>06 11 82 71 28</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1300,17 +1300,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Stéphanie Chissadon - Optimhome</t>
+          <t>Véronique Mondon - iad France</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Stéphanie Chissadon</t>
+          <t>Véronique Mondon</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>06 85 02 76 46</t>
+          <t>06 77 92 28 12</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1322,22 +1322,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Théau Silbermann</t>
+          <t>Aurelien CENCI - IAD France</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Théau Silbermann</t>
+          <t>Aurélien Cenci</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>06 11 82 71 28</t>
+          <t>06 26 44 64 05</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1349,22 +1349,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Véronique Mondon - iad France</t>
+          <t>Delaporte Immobilier</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Véronique Mondon</t>
+          <t>Aurélien Delaporte</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>06 77 92 28 12</t>
+          <t>06 19 48 20 93</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1381,17 +1381,17 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Aurelien CENCI - IAD France</t>
+          <t>e-mobilier Amiens</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Aurélien Cenci</t>
+          <t>S. Benarous (agent)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>06 26 44 64 05</t>
+          <t>06 35 22 43 99</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -1408,17 +1408,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Delaporte Immobilier</t>
+          <t>ESPACE &amp; WALL</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Aurélien Delaporte</t>
+          <t>Émilie Wolinne (Présidente)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>06 19 48 20 93</t>
+          <t>06 85 72 68 51</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>e-mobilier Amiens</t>
+          <t>Foudhil DAOUDI - EXPERTIMO</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>S. Benarous (agent)</t>
+          <t>Foudhil Daoudi</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>06 35 22 43 99</t>
+          <t>06 64 16 11 21</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -1462,17 +1462,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ESPACE &amp; WALL</t>
+          <t>Gregory Mattens (BSK Immobilier)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Émilie Wolinne (Présidente)</t>
+          <t>Gregory Mattens</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>06 85 72 68 51</t>
+          <t>06 63 69 65 00</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -1489,17 +1489,17 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Estelle Desnain - Conseiller immobilier</t>
+          <t>Hugo DUFOUR - iad Immobilier</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Estelle Desnain</t>
+          <t>Hugo Dufour</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>06 10 93 58 83</t>
+          <t>06 25 82 22 60</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -1516,17 +1516,17 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Foudhil DAOUDI - EXPERTIMO</t>
+          <t>Isabelle BOHAIN - IAD France</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Foudhil Daoudi</t>
+          <t>Isabelle Bohain</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>06 64 16 11 21</t>
+          <t>06 69 51 10 53</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -1543,17 +1543,17 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Gregory Mattens (BSK Immobilier)</t>
+          <t>Jérôme BAILLET - IAD France</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Gregory Mattens</t>
+          <t>Jérôme Baillet</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>06 63 69 65 00</t>
+          <t>06 81 42 56 26</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Hugo DUFOUR - iad Immobilier</t>
+          <t>Quinet Nicolas</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Hugo Dufour</t>
+          <t>Nicolas Quinet</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>06 25 82 22 60</t>
+          <t>06 28 74 00 81</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Isabelle BOHAIN - IAD France</t>
+          <t>Stéphane DEBEAUVAIS - IAD</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Isabelle Bohain</t>
+          <t>Stéphane Debeauvais</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>06 69 51 10 53</t>
+          <t>06 21 38 83 15</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Jérôme BAILLET - IAD France</t>
+          <t>Sylvie Dieu - IAD France</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Jérôme Baillet</t>
+          <t>Sylvie Dieu</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>06 81 42 56 26</t>
+          <t>07 81 31 35 43</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -1651,17 +1651,17 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Quinet Nicolas</t>
+          <t>VERDIER Immobilier (Le Centre Immobilier)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Nicolas Quinet</t>
+          <t>Nicolas Verdier</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>06 28 74 00 81</t>
+          <t>06 75 21 21 69</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -1673,130 +1673,130 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Sophie Hardy Immobilier</t>
+          <t>Agence immobilière 360° à Angers</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Sophie Hardy</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>06 79 07 80 19</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 12 66 56 83</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Stéphane DEBEAUVAIS - IAD</t>
+          <t>Le bon agent immobilier Angers</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Stéphane Debeauvais</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>06 21 38 83 15</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 11 51 51 87</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Sylvie Dieu - IAD France</t>
+          <t>SDSIMMO L'AGENCE</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Sylvie Dieu</t>
+          <t>Antoine Fauché (Président)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>07 81 31 35 43</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 77 25 24 83</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>VERDIER Immobilier (Le Centre Immobilier)</t>
+          <t>Agence ICImmobilier</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Nicolas Verdier</t>
+          <t>Jean-Marc Eisenbach</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>06 75 21 21 69</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
+          <t>06 87 45 16 27</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Non précisé</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Agence immobilière 360° à Angers</t>
+          <t>Agence Pascale Louis Immobilier</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Pascale Louis</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>06 12 66 56 83</t>
+          <t>06 07 25 76 74</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -1808,22 +1808,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Le bon agent immobilier Angers</t>
+          <t>Logimmo Conseil</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Aurélie Bernardet</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>06 11 51 51 87</t>
+          <t>06 52 49 18 58</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -1835,22 +1835,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>SDSIMMO L'AGENCE</t>
+          <t>Manada Immobilier</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Antoine Fauché (Président)</t>
+          <t>Marine &amp; Julie Fananas</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>06 77 25 24 83</t>
+          <t>06 58 04 00 29</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -1862,22 +1862,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Agence ICImmobilier</t>
+          <t>Immo en Somme</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Jean-Marc Eisenbach</t>
+          <t>Anthony Mortas</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>06 87 45 16 27</t>
+          <t>06 15 01 61 62</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -1889,22 +1889,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Agence Pascale Louis Immobilier</t>
+          <t>Josse Pelletier Immobilier</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Pascale Louis</t>
+          <t>Sébastien Josse &amp; Isabelle Pelletier</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>06 07 25 76 74</t>
+          <t>06 67 27 80 80</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -1916,22 +1916,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Logimmo Conseil</t>
+          <t>Toit pour toi</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Aurélie Bernardet</t>
+          <t>Michel Amarens</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>06 52 49 18 58</t>
+          <t>07 67 07 19 08</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -1943,93 +1943,93 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Manada Immobilier</t>
+          <t>IMMO PROFESSIONNEL</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Marine &amp; Julie Fananas</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>06 58 04 00 29</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 52 52 58 84</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Immo en Somme</t>
+          <t>Sylvain - Les Arènes Immobilier</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Anthony Mortas</t>
+          <t>Sylvain (négociateur)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>06 15 01 61 62</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 62 95 93 80</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Josse Pelletier Immobilier</t>
+          <t>Agence Estia Immobilier</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Sébastien Josse &amp; Isabelle Pelletier</t>
+          <t>Caroline Florance</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>06 67 27 80 80</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 63 79 66 76</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Satisfimmo</t>
+          <t>HOME</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2039,61 +2039,61 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>06 15 35 62 54</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 07 49 43 37</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Toit pour toi</t>
+          <t>AAlivImmo (A. Alivi Immo)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Michel Amarens</t>
+          <t>Non identifié sur Pappers</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>07 67 07 19 08</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Non précisé</t>
+          <t>06 19 77 10 66</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>IMMO PROFESSIONNEL</t>
+          <t>Agence La Locale Limoges</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Julien Ribierre &amp; Dylan Di Nato</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>06 52 52 58 84</t>
+          <t>06 12 19 81 65</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -2105,22 +2105,22 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Sylvain - Les Arènes Immobilier</t>
+          <t>Julien Beauzetier (La Halle de l'Immobilier)</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Sylvain (négociateur)</t>
+          <t>Julien Beauzetier</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>06 62 95 93 80</t>
+          <t>06 11 09 74 89</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -2132,22 +2132,22 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Agence Estia Immobilier</t>
+          <t>Nouveaux Horizons - Immobilier</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Caroline Florance</t>
+          <t>Romain Bardon</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>06 63 79 66 76</t>
+          <t>06 17 86 76 26</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
@@ -2159,22 +2159,22 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Limoges</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>ROMAIN TERRAL</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Romain Terral</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>06 07 49 43 37</t>
+          <t>06 40 92 22 95</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>AAlivImmo (A. Alivi Immo)</t>
+          <t>Véronique QUEYREIX</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Non identifié sur Pappers</t>
+          <t>Véronique Queyreix</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>06 19 77 10 66</t>
+          <t>06 20 88 58 23</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
@@ -2213,22 +2213,22 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Agence La Locale Limoges</t>
+          <t>Cabinet Immobilier Amiénois</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Julien Ribierre &amp; Dylan Di Nato</t>
+          <t>Romain Hecquet (Président)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>06 12 19 81 65</t>
+          <t>06 24 21 58 52</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
@@ -2240,22 +2240,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Julien Beauzetier (La Halle de l'Immobilier)</t>
+          <t>HAUTS DE FRANCE IMMOBILIER</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Julien Beauzetier</t>
+          <t>Lilian Cléry (Président)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>06 11 09 74 89</t>
+          <t>06 08 51 24 30</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -2267,22 +2267,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Limoges</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Mélodie Garcia - La Halle de l'Immobilier</t>
+          <t>SNG Amiens</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Mélodie Garcia</t>
+          <t>Jérôme Vangrevelynghe (conseiller)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>06 95 70 17 07</t>
+          <t>06 79 22 09 64</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -2291,170 +2291,8 @@
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>Nouveaux Horizons - Immobilier</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Romain Bardon</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>06 17 86 76 26</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>ROMAIN TERRAL</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>Romain Terral</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>06 40 92 22 95</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Limoges</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>Véronique QUEYREIX</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>Véronique Queyreix</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>06 20 88 58 23</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>Cabinet Immobilier Amiénois</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>Romain Hecquet (Président)</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>06 24 21 58 52</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>HAUTS DE FRANCE IMMOBILIER</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>Lilian Cléry (Président)</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>06 08 51 24 30</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Amiens</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>SNG Amiens</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>Jérôme Vangrevelynghe (conseiller)</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>06 79 22 09 64</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E73"/>
+  <autoFilter ref="A1:E67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>